<commit_message>
Marca Camisa JC 5 como agotada
</commit_message>
<xml_diff>
--- a/productos.xlsx
+++ b/productos.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +32,10 @@
     <font>
       <b val="1"/>
       <color rgb="00F5F5F5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
     </font>
   </fonts>
   <fills count="3">
@@ -59,7 +63,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -69,6 +73,9 @@
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -624,8 +631,8 @@
         <v>120000</v>
       </c>
       <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="2" t="n">
-        <v>5</v>
+      <c r="G6" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
     </row>

</xml_diff>